<commit_message>
feat: integrate workflow daily orchestration and governance
</commit_message>
<xml_diff>
--- a/test-data/tenant-config-packages/tb-tenant-config-package-test.xlsx
+++ b/test-data/tenant-config-packages/tb-tenant-config-package-test.xlsx
@@ -1847,7 +1847,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>{"url":"http://mockserver:1080/tb/callback","method":"POST","tokenHeader":"X-API-Token"}</t>
+          <t>{"target_endpoint":"http://mockserver:1080/tb/callback"}</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>{"url": "http://mockserver:1080/tb/ingest", "method": "POST", "tokenHeader": "X-API-Token", "target_endpoint": "http://mockserver:1080/tb/ingest"}</t>
+          <t>{"target_endpoint":"http://mockserver:1080/tb/ingest"}</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>